<commit_message>
Drop west coast; Tasman glacier hike from Mount Cook Village
Skip Hokitika/Franz Josef. Stay three nights in Mount Cook Village
for the Tasman heli-hike, then linger at Pukaki before Arrowtown.

Co-authored-by: max123465 <max123465@users.noreply.github.com>
</commit_message>
<xml_diff>
--- a/travel/nz-south-island-chill-2027apr/NZ_South_Island_chill_2pax_2027apr.xlsx
+++ b/travel/nz-south-island-chill-2027apr/NZ_South_Island_chill_2pax_2027apr.xlsx
@@ -675,7 +675,7 @@
     <row r="5" ht="22" customHeight="1">
       <c r="A5" s="2" t="inlineStr">
         <is>
-          <t>3. 橘色列是長途或看天氣的日子：4/20 西岸、4/22 冰川、4/24 Haast、4/28 米佛、4/29 回麥肯齊。</t>
+          <t>3. 橘色列是長途或看天氣的日子：4/20 凱庫拉到蒂卡波、4/23 冰川、5/1 米佛、5/2 回蒂卡波。</t>
         </is>
       </c>
     </row>
@@ -1067,7 +1067,7 @@
     <row r="22">
       <c r="A22" s="11" t="inlineStr">
         <is>
-          <t>活動（表內 5 項）</t>
+          <t>活動（表內 4 項）</t>
         </is>
       </c>
       <c r="B22" s="12">
@@ -1084,7 +1084,7 @@
       </c>
       <c r="E22" s="11" t="inlineStr">
         <is>
-          <t>賞鯨＋冰川＋米佛＋探險＋觀星</t>
+          <t>賞鯨＋塔斯曼冰川健行＋米佛＋觀星</t>
         </is>
       </c>
     </row>
@@ -1172,14 +1172,14 @@
     <row r="29" ht="32" customHeight="1">
       <c r="A29" s="2" t="inlineStr">
         <is>
-          <t>路線改 chill：凱庫拉 2 晚、弗蘭茲 3 晚、箭鎮 3 晚、普卡基＋蒂卡波 4 晚。砍皮克頓、但尼丁、奧瑪魯。</t>
+          <t>不走西岸。冰川改在庫克山村做塔斯曼 heli-hike。凱庫拉 2 晚、麥肯齊 8 晚、箭鎮 3 晚。</t>
         </is>
       </c>
     </row>
     <row r="30" ht="32" customHeight="1">
       <c r="A30" s="2" t="inlineStr">
         <is>
-          <t>箭鎮 4 月下旬是金黃季。2027 Autumn Festival 是 4/15–18，你們 4/24 才到，人較少、葉子通常還在。</t>
+          <t>箭鎮改住 4/27–29，仍在金黃窗口。2027 秋祭是 4/15–18，你們會錯過人潮。</t>
         </is>
       </c>
     </row>
@@ -1536,38 +1536,38 @@
       </c>
       <c r="D6" s="32" t="inlineStr">
         <is>
-          <t>霍基蒂卡</t>
+          <t>蒂卡波</t>
         </is>
       </c>
       <c r="E6" s="33" t="inlineStr">
         <is>
-          <t>經 Hanmer＋Lewis Pass 6.5h</t>
+          <t>Kaikoura→Tekapo 6h</t>
         </is>
       </c>
       <c r="F6" s="34" t="n">
-        <v>420</v>
+        <v>450</v>
       </c>
       <c r="G6" s="33" t="inlineStr">
         <is>
-          <t>經漢默泉泡湯 1.5–2h（不必過夜），再走 Lewis Pass 到西岸。夠力再停 Pancake Rocks。</t>
+          <t>原路回 SH1 南下，經 Geraldine、Fairlie 進麥肯齊。傍晚牧羊人教堂。不繞西岸。</t>
         </is>
       </c>
       <c r="H6" s="33" t="inlineStr">
         <is>
-          <t>漢默泉泡湯（可選）</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I6" s="23" t="n">
-        <v>80</v>
+        <v>0</v>
       </c>
       <c r="J6" s="23" t="n">
-        <v>140</v>
+        <v>230</v>
       </c>
       <c r="K6" s="23" t="n">
         <v>130</v>
       </c>
       <c r="L6" s="23" t="n">
-        <v>90</v>
+        <v>96</v>
       </c>
       <c r="M6" s="35">
         <f>('01_總覽'!$B$8+'01_總覽'!$B$9)</f>
@@ -1583,7 +1583,7 @@
       </c>
       <c r="P6" s="33" t="inlineStr">
         <is>
-          <t>Hokitika motel｜全行程最長車日。漢默泡湯當中途休息。沿路加油。</t>
+          <t>湖景 motel；無景房不值得｜這天是最長車日。中午在 Geraldine 吃飯休息。</t>
         </is>
       </c>
     </row>
@@ -1603,38 +1603,38 @@
       </c>
       <c r="D7" s="21" t="inlineStr">
         <is>
-          <t>弗蘭茲約瑟夫</t>
+          <t>蒂卡波</t>
         </is>
       </c>
       <c r="E7" s="11" t="inlineStr">
         <is>
-          <t>Hokitika→Franz 2h</t>
+          <t>當地</t>
         </is>
       </c>
       <c r="F7" s="22" t="n">
-        <v>160</v>
+        <v>25</v>
       </c>
       <c r="G7" s="11" t="inlineStr">
         <is>
-          <t>上午 Hokitika Gorge（免費、水色很美）。午後抵冰川村報到、走谷底步道遠看冰。</t>
+          <t>整天留著。教堂日出、湖邊、Tekapo Springs。晚上 Dark Sky 約翰山。</t>
         </is>
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Dark Sky 約翰山 Summit</t>
         </is>
       </c>
       <c r="I7" s="23" t="n">
-        <v>0</v>
+        <v>478</v>
       </c>
       <c r="J7" s="23" t="n">
-        <v>180</v>
+        <v>230</v>
       </c>
       <c r="K7" s="23" t="n">
         <v>130</v>
       </c>
       <c r="L7" s="23" t="n">
-        <v>35</v>
+        <v>6</v>
       </c>
       <c r="M7" s="12">
         <f>('01_總覽'!$B$8+'01_總覽'!$B$9)</f>
@@ -1650,177 +1650,177 @@
       </c>
       <c r="P7" s="11" t="inlineStr">
         <is>
-          <t>Franz 中價 motel｜Heli-hike 明天。今天只適應西岸天氣。</t>
+          <t>連住第 2 晚｜Summit 約 NZ$219–239。觀星看雲，有室內備援。</t>
         </is>
       </c>
     </row>
     <row r="8" ht="48" customHeight="1">
-      <c r="A8" s="31" t="n">
+      <c r="A8" s="25" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="32" t="inlineStr">
+      <c r="B8" s="7" t="inlineStr">
         <is>
           <t>2027/4/22</t>
         </is>
       </c>
-      <c r="C8" s="32" t="inlineStr">
+      <c r="C8" s="7" t="inlineStr">
         <is>
           <t>四</t>
         </is>
       </c>
-      <c r="D8" s="32" t="inlineStr">
-        <is>
-          <t>弗蘭茲約瑟夫</t>
-        </is>
-      </c>
-      <c r="E8" s="33" t="inlineStr">
+      <c r="D8" s="7" t="inlineStr">
+        <is>
+          <t>庫克山村</t>
+        </is>
+      </c>
+      <c r="E8" s="26" t="inlineStr">
+        <is>
+          <t>Tekapo→Mt Cook 1.5h</t>
+        </is>
+      </c>
+      <c r="F8" s="27" t="n">
+        <v>105</v>
+      </c>
+      <c r="G8" s="26" t="inlineStr">
+        <is>
+          <t>經普卡基牛奶藍進村。下午走免費 Tasman Glacier View（車 10 分＋步道 40 分）。報到冰川健行。</t>
+        </is>
+      </c>
+      <c r="H8" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
+        </is>
+      </c>
+      <c r="I8" s="23" t="n">
+        <v>0</v>
+      </c>
+      <c r="J8" s="23" t="n">
+        <v>320</v>
+      </c>
+      <c r="K8" s="23" t="n">
+        <v>150</v>
+      </c>
+      <c r="L8" s="23" t="n">
+        <v>24</v>
+      </c>
+      <c r="M8" s="28">
+        <f>('01_總覽'!$B$8+'01_總覽'!$B$9)</f>
+        <v/>
+      </c>
+      <c r="N8" s="29">
+        <f>I8+J8+K8+L8+M8</f>
+        <v/>
+      </c>
+      <c r="O8" s="30">
+        <f>N8*'01_總覽'!$B$5</f>
+        <v/>
+      </c>
+      <c r="P8" s="26" t="inlineStr">
+        <is>
+          <t>隱士山景或 Aoraki Court｜塔斯曼冰川就在村外，不用去弗蘭茲。隱士無景房不值得。</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="48" customHeight="1">
+      <c r="A9" s="31" t="n">
+        <v>7</v>
+      </c>
+      <c r="B9" s="32" t="inlineStr">
+        <is>
+          <t>2027/4/23</t>
+        </is>
+      </c>
+      <c r="C9" s="32" t="inlineStr">
+        <is>
+          <t>五</t>
+        </is>
+      </c>
+      <c r="D9" s="32" t="inlineStr">
+        <is>
+          <t>庫克山村</t>
+        </is>
+      </c>
+      <c r="E9" s="33" t="inlineStr">
+        <is>
+          <t>當地／機場 10 分</t>
+        </is>
+      </c>
+      <c r="F9" s="34" t="n">
+        <v>20</v>
+      </c>
+      <c r="G9" s="33" t="inlineStr">
+        <is>
+          <t>塔斯曼冰川健行：庫克山機場集合，直升機上冰走約 2 小時。取消則改 4/24。</t>
+        </is>
+      </c>
+      <c r="H9" s="33" t="inlineStr">
+        <is>
+          <t>Tasman Glacier heli-hike</t>
+        </is>
+      </c>
+      <c r="I9" s="23" t="n">
+        <v>1990</v>
+      </c>
+      <c r="J9" s="23" t="n">
+        <v>320</v>
+      </c>
+      <c r="K9" s="23" t="n">
+        <v>150</v>
+      </c>
+      <c r="L9" s="23" t="n">
+        <v>6</v>
+      </c>
+      <c r="M9" s="35">
+        <f>('01_總覽'!$B$8+'01_總覽'!$B$9)</f>
+        <v/>
+      </c>
+      <c r="N9" s="36">
+        <f>I9+J9+K9+L9+M9</f>
+        <v/>
+      </c>
+      <c r="O9" s="37">
+        <f>N9*'01_總覽'!$B$5</f>
+        <v/>
+      </c>
+      <c r="P9" s="33" t="inlineStr">
+        <is>
+          <t>連住｜Alpine Guides／Mt Cook Glacier Guiding 約 NZ$995／人，至 2027/9/30。在庫克山機場出發。</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="48" customHeight="1">
+      <c r="A10" s="25" t="n">
+        <v>8</v>
+      </c>
+      <c r="B10" s="7" t="inlineStr">
+        <is>
+          <t>2027/4/24</t>
+        </is>
+      </c>
+      <c r="C10" s="7" t="inlineStr">
+        <is>
+          <t>六</t>
+        </is>
+      </c>
+      <c r="D10" s="7" t="inlineStr">
+        <is>
+          <t>庫克山村</t>
+        </is>
+      </c>
+      <c r="E10" s="26" t="inlineStr">
         <is>
           <t>當地</t>
         </is>
       </c>
-      <c r="F8" s="34" t="n">
-        <v>20</v>
-      </c>
-      <c r="G8" s="33" t="inlineStr">
-        <is>
-          <t>直升機冰川健行（半天，裝備全含）。取消則改 4/23。下午回房休息。</t>
-        </is>
-      </c>
-      <c r="H8" s="33" t="inlineStr">
-        <is>
-          <t>Franz heli-hike</t>
-        </is>
-      </c>
-      <c r="I8" s="23" t="n">
-        <v>1798</v>
-      </c>
-      <c r="J8" s="23" t="n">
-        <v>180</v>
-      </c>
-      <c r="K8" s="23" t="n">
-        <v>130</v>
-      </c>
-      <c r="L8" s="23" t="n">
-        <v>6</v>
-      </c>
-      <c r="M8" s="35">
-        <f>('01_總覽'!$B$8+'01_總覽'!$B$9)</f>
-        <v/>
-      </c>
-      <c r="N8" s="36">
-        <f>I8+J8+K8+L8+M8</f>
-        <v/>
-      </c>
-      <c r="O8" s="37">
-        <f>N8*'01_總覽'!$B$5</f>
-        <v/>
-      </c>
-      <c r="P8" s="33" t="inlineStr">
-        <is>
-          <t>連住｜官網至 2027/9/30 為 NZ$899／人。西岸取消率高，所以連住 3 晚。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9" ht="48" customHeight="1">
-      <c r="A9" s="20" t="n">
-        <v>7</v>
-      </c>
-      <c r="B9" s="21" t="inlineStr">
-        <is>
-          <t>2027/4/23</t>
-        </is>
-      </c>
-      <c r="C9" s="21" t="inlineStr">
-        <is>
-          <t>五</t>
-        </is>
-      </c>
-      <c r="D9" s="21" t="inlineStr">
-        <is>
-          <t>弗蘭茲約瑟夫</t>
-        </is>
-      </c>
-      <c r="E9" s="11" t="inlineStr">
-        <is>
-          <t>Franz↔Fox 往返</t>
-        </is>
-      </c>
-      <c r="F9" s="22" t="n">
-        <v>50</v>
-      </c>
-      <c r="G9" s="11" t="inlineStr">
-        <is>
-          <t>天氣備援日。能飛就補 heli-hike；不能就黎明去 Lake Matheson 拍鏡面。整天可以很閒。</t>
-        </is>
-      </c>
-      <c r="H9" s="11" t="inlineStr">
-        <is>
-          <t>—</t>
-        </is>
-      </c>
-      <c r="I9" s="23" t="n">
-        <v>0</v>
-      </c>
-      <c r="J9" s="23" t="n">
-        <v>180</v>
-      </c>
-      <c r="K9" s="23" t="n">
-        <v>130</v>
-      </c>
-      <c r="L9" s="23" t="n">
-        <v>12</v>
-      </c>
-      <c r="M9" s="12">
-        <f>('01_總覽'!$B$8+'01_總覽'!$B$9)</f>
-        <v/>
-      </c>
-      <c r="N9" s="24">
-        <f>I9+J9+K9+L9+M9</f>
-        <v/>
-      </c>
-      <c r="O9" s="13">
-        <f>N9*'01_總覽'!$B$5</f>
-        <v/>
-      </c>
-      <c r="P9" s="11" t="inlineStr">
-        <is>
-          <t>連住第 3 晚｜這晚是為冰川天氣買的保險，不要再往前趕。</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="48" customHeight="1">
-      <c r="A10" s="31" t="n">
-        <v>8</v>
-      </c>
-      <c r="B10" s="32" t="inlineStr">
-        <is>
-          <t>2027/4/24</t>
-        </is>
-      </c>
-      <c r="C10" s="32" t="inlineStr">
-        <is>
-          <t>六</t>
-        </is>
-      </c>
-      <c r="D10" s="32" t="inlineStr">
-        <is>
-          <t>箭鎮</t>
-        </is>
-      </c>
-      <c r="E10" s="33" t="inlineStr">
-        <is>
-          <t>Franz→Haast→Wanaka→Arrowtown 5h</t>
-        </is>
-      </c>
-      <c r="F10" s="34" t="n">
-        <v>400</v>
-      </c>
-      <c r="G10" s="33" t="inlineStr">
-        <is>
-          <t>Haast Pass 本身是景。Wanaka 咖啡＋That Wanaka Tree。傍晚進箭鎮住下來。</t>
-        </is>
-      </c>
-      <c r="H10" s="33" t="inlineStr">
+      <c r="F10" s="27" t="n">
+        <v>25</v>
+      </c>
+      <c r="G10" s="26" t="inlineStr">
+        <is>
+          <t>天氣備援日。能飛就補健行；不能就走 Hooker Valley。想坐冰河湖船再加 Glacier Explorers。</t>
+        </is>
+      </c>
+      <c r="H10" s="26" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -1829,29 +1829,29 @@
         <v>0</v>
       </c>
       <c r="J10" s="23" t="n">
-        <v>230</v>
+        <v>320</v>
       </c>
       <c r="K10" s="23" t="n">
-        <v>140</v>
+        <v>150</v>
       </c>
       <c r="L10" s="23" t="n">
-        <v>85</v>
-      </c>
-      <c r="M10" s="35">
+        <v>6</v>
+      </c>
+      <c r="M10" s="28">
         <f>('01_總覽'!$B$8+'01_總覽'!$B$9)</f>
         <v/>
       </c>
-      <c r="N10" s="36">
+      <c r="N10" s="29">
         <f>I10+J10+K10+L10+M10</f>
         <v/>
       </c>
-      <c r="O10" s="37">
+      <c r="O10" s="30">
         <f>N10*'01_總覽'!$B$5</f>
         <v/>
       </c>
-      <c r="P10" s="33" t="inlineStr">
-        <is>
-          <t>箭鎮村內 B&amp;B／motel，不要住皇后鎮｜Haast 前加油。週六箭鎮較擠，先入住，楓葉留明天清晨。</t>
+      <c r="P10" s="26" t="inlineStr">
+        <is>
+          <t>連住第 3 晚｜這晚是為冰川天氣買的保險。船是另一件事，不是走上冰。</t>
         </is>
       </c>
     </row>
@@ -1871,20 +1871,20 @@
       </c>
       <c r="D11" s="21" t="inlineStr">
         <is>
-          <t>箭鎮</t>
+          <t>普卡基／Twizel</t>
         </is>
       </c>
       <c r="E11" s="11" t="inlineStr">
         <is>
-          <t>當地／Lake Hayes</t>
+          <t>Mt Cook→Pukaki 50min</t>
         </is>
       </c>
       <c r="F11" s="22" t="n">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="G11" s="11" t="inlineStr">
         <is>
-          <t>07:30 前走 Buckingham Street、中國村、Arrow River。再到 Lake Hayes 拍倒影。下午發呆。</t>
+          <t>早上 Hooker Valley（若昨天沒走）。慢慢開到普卡基看牛奶藍，下午發呆。</t>
         </is>
       </c>
       <c r="H11" s="11" t="inlineStr">
@@ -1896,13 +1896,13 @@
         <v>0</v>
       </c>
       <c r="J11" s="23" t="n">
-        <v>230</v>
+        <v>200</v>
       </c>
       <c r="K11" s="23" t="n">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="L11" s="23" t="n">
-        <v>10</v>
+        <v>16</v>
       </c>
       <c r="M11" s="12">
         <f>('01_總覽'!$B$8+'01_總覽'!$B$9)</f>
@@ -1918,7 +1918,7 @@
       </c>
       <c r="P11" s="11" t="inlineStr">
         <is>
-          <t>連住｜4 月下旬是箭鎮金黃高峰。主要是楊樹、橡樹、楓香，不是台灣那種楓。</t>
+          <t>普卡基湖景 cabin 或 Twizel motel｜Twizel 有超市。湖景訂普卡基路邊。</t>
         </is>
       </c>
     </row>
@@ -1938,20 +1938,20 @@
       </c>
       <c r="D12" s="7" t="inlineStr">
         <is>
-          <t>箭鎮</t>
+          <t>普卡基／Twizel</t>
         </is>
       </c>
       <c r="E12" s="26" t="inlineStr">
         <is>
-          <t>可去皇后鎮或 Glenorchy</t>
+          <t>當地</t>
         </is>
       </c>
       <c r="F12" s="27" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="G12" s="26" t="inlineStr">
         <is>
-          <t>週一比較空。可去 Glenorchy 湖灣，或皇后鎮散步。不跳傘、不彈跳。酒莊要有指定駕駛。</t>
+          <t>整天留著。日出看庫克山、沿湖散步。不想開車就待著。</t>
         </is>
       </c>
       <c r="H12" s="26" t="inlineStr">
@@ -1963,13 +1963,13 @@
         <v>0</v>
       </c>
       <c r="J12" s="23" t="n">
-        <v>230</v>
+        <v>200</v>
       </c>
       <c r="K12" s="23" t="n">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="L12" s="23" t="n">
-        <v>18</v>
+        <v>10</v>
       </c>
       <c r="M12" s="28">
         <f>('01_總覽'!$B$8+'01_總覽'!$B$9)</f>
@@ -1985,7 +1985,7 @@
       </c>
       <c r="P12" s="26" t="inlineStr">
         <is>
-          <t>連住第 3 晚｜Arrowtown Autumn Festival 是 4/15–18，你們會錯過人潮，楓葉通常還在。</t>
+          <t>連住第 2 晚｜這兩晚就是你們要的普卡基久住。</t>
         </is>
       </c>
     </row>
@@ -2005,38 +2005,38 @@
       </c>
       <c r="D13" s="21" t="inlineStr">
         <is>
-          <t>蒂阿瑙</t>
+          <t>箭鎮</t>
         </is>
       </c>
       <c r="E13" s="11" t="inlineStr">
         <is>
-          <t>Arrowtown→Te Anau 2.5h</t>
+          <t>Pukaki→Lindis→Arrowtown 4h</t>
         </is>
       </c>
       <c r="F13" s="22" t="n">
-        <v>190</v>
+        <v>280</v>
       </c>
       <c r="G13" s="11" t="inlineStr">
         <is>
-          <t>中午前出發即可。超市補米佛隔日食物（沿路沒店）。晚上想去再訂螢火蟲洞，不勉強。</t>
+          <t>經 Omarama、Lindis Pass、Cromwell。Wanaka 想停就停。傍晚進箭鎮。</t>
         </is>
       </c>
       <c r="H13" s="11" t="inlineStr">
         <is>
-          <t>螢火蟲洞（可選，表內未列）</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I13" s="23" t="n">
         <v>0</v>
       </c>
       <c r="J13" s="23" t="n">
-        <v>180</v>
+        <v>230</v>
       </c>
       <c r="K13" s="23" t="n">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="L13" s="23" t="n">
-        <v>42</v>
+        <v>60</v>
       </c>
       <c r="M13" s="12">
         <f>('01_總覽'!$B$8+'01_總覽'!$B$9)</f>
@@ -2052,141 +2052,141 @@
       </c>
       <c r="P13" s="11" t="inlineStr">
         <is>
-          <t>Distinction / Lakefront｜螢火蟲洞約 NZ$145–154／人。累了就看湖。</t>
+          <t>箭鎮村內，不要住皇后鎮｜Lindis 秋天很美。Omarama 可選熱湯池。</t>
         </is>
       </c>
     </row>
     <row r="14" ht="48" customHeight="1">
-      <c r="A14" s="31" t="n">
+      <c r="A14" s="25" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="32" t="inlineStr">
+      <c r="B14" s="7" t="inlineStr">
         <is>
           <t>2027/4/28</t>
         </is>
       </c>
-      <c r="C14" s="32" t="inlineStr">
+      <c r="C14" s="7" t="inlineStr">
         <is>
           <t>三</t>
         </is>
       </c>
-      <c r="D14" s="32" t="inlineStr">
-        <is>
-          <t>蒂阿瑙</t>
-        </is>
-      </c>
-      <c r="E14" s="33" t="inlineStr">
-        <is>
-          <t>Te Anau↔Milford 往返 5h</t>
-        </is>
-      </c>
-      <c r="F14" s="34" t="n">
-        <v>240</v>
-      </c>
-      <c r="G14" s="33" t="inlineStr">
-        <is>
-          <t>07:00 自駕 SH94：Mirror Lakes、Homer Tunnel。訂 11:10 或 13:30 小船。傍晚回蒂阿瑙。</t>
-        </is>
-      </c>
-      <c r="H14" s="33" t="inlineStr">
-        <is>
-          <t>米佛峽灣遊船（自駕＋船）</t>
+      <c r="D14" s="7" t="inlineStr">
+        <is>
+          <t>箭鎮</t>
+        </is>
+      </c>
+      <c r="E14" s="26" t="inlineStr">
+        <is>
+          <t>當地／Lake Hayes</t>
+        </is>
+      </c>
+      <c r="F14" s="27" t="n">
+        <v>40</v>
+      </c>
+      <c r="G14" s="26" t="inlineStr">
+        <is>
+          <t>07:30 前走 Buckingham Street、中國村、Arrow River。再到 Lake Hayes。</t>
+        </is>
+      </c>
+      <c r="H14" s="26" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="I14" s="23" t="n">
-        <v>376</v>
+        <v>0</v>
       </c>
       <c r="J14" s="23" t="n">
-        <v>180</v>
+        <v>230</v>
       </c>
       <c r="K14" s="23" t="n">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="L14" s="23" t="n">
-        <v>52</v>
-      </c>
-      <c r="M14" s="35">
+        <v>10</v>
+      </c>
+      <c r="M14" s="28">
         <f>('01_總覽'!$B$8+'01_總覽'!$B$9)</f>
         <v/>
       </c>
-      <c r="N14" s="36">
+      <c r="N14" s="29">
         <f>I14+J14+K14+L14+M14</f>
         <v/>
       </c>
-      <c r="O14" s="37">
+      <c r="O14" s="30">
         <f>N14*'01_總覽'!$B$5</f>
         <v/>
       </c>
-      <c r="P14" s="33" t="inlineStr">
-        <is>
-          <t>連住｜Mitre Peak／Cruise Milford 約 NZ$179–188。不要買皇后鎮巴士一日遊。</t>
+      <c r="P14" s="26" t="inlineStr">
+        <is>
+          <t>連住｜4 月底仍是金黃窗口。主要是楊樹、橡樹、楓香。</t>
         </is>
       </c>
     </row>
     <row r="15" ht="48" customHeight="1">
-      <c r="A15" s="31" t="n">
+      <c r="A15" s="20" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="32" t="inlineStr">
+      <c r="B15" s="21" t="inlineStr">
         <is>
           <t>2027/4/29</t>
         </is>
       </c>
-      <c r="C15" s="32" t="inlineStr">
+      <c r="C15" s="21" t="inlineStr">
         <is>
           <t>四</t>
         </is>
       </c>
-      <c r="D15" s="32" t="inlineStr">
-        <is>
-          <t>普卡基／Twizel</t>
-        </is>
-      </c>
-      <c r="E15" s="33" t="inlineStr">
-        <is>
-          <t>經 Cromwell＋Lindis 6h</t>
-        </is>
-      </c>
-      <c r="F15" s="34" t="n">
-        <v>400</v>
-      </c>
-      <c r="G15" s="33" t="inlineStr">
-        <is>
-          <t>回程不繞但尼丁。Lindis Pass 秋天很美。Omarama 可停熱湯池。傍晚抵普卡基看牛奶藍。</t>
-        </is>
-      </c>
-      <c r="H15" s="33" t="inlineStr">
-        <is>
-          <t>Omarama Hot Tubs（可選）</t>
+      <c r="D15" s="21" t="inlineStr">
+        <is>
+          <t>箭鎮</t>
+        </is>
+      </c>
+      <c r="E15" s="11" t="inlineStr">
+        <is>
+          <t>可去 Glenorchy</t>
+        </is>
+      </c>
+      <c r="F15" s="22" t="n">
+        <v>80</v>
+      </c>
+      <c r="G15" s="11" t="inlineStr">
+        <is>
+          <t>人少的一天。Glenorchy 湖灣或皇后鎮散步。不跳傘。</t>
+        </is>
+      </c>
+      <c r="H15" s="11" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="I15" s="23" t="n">
         <v>0</v>
       </c>
       <c r="J15" s="23" t="n">
-        <v>200</v>
+        <v>230</v>
       </c>
       <c r="K15" s="23" t="n">
-        <v>130</v>
+        <v>140</v>
       </c>
       <c r="L15" s="23" t="n">
-        <v>85</v>
-      </c>
-      <c r="M15" s="35">
+        <v>18</v>
+      </c>
+      <c r="M15" s="12">
         <f>('01_總覽'!$B$8+'01_總覽'!$B$9)</f>
         <v/>
       </c>
-      <c r="N15" s="36">
+      <c r="N15" s="24">
         <f>I15+J15+K15+L15+M15</f>
         <v/>
       </c>
-      <c r="O15" s="37">
+      <c r="O15" s="13">
         <f>N15*'01_總覽'!$B$5</f>
         <v/>
       </c>
-      <c r="P15" s="33" t="inlineStr">
-        <is>
-          <t>普卡基湖景 cabin 或 Twizel motel｜Twizel 有超市、比較好住；湖景要訂普卡基路邊。</t>
+      <c r="P15" s="11" t="inlineStr">
+        <is>
+          <t>連住第 3 晚｜秋祭是 4/15–18，這幾天人比較少。</t>
         </is>
       </c>
     </row>
@@ -2206,38 +2206,38 @@
       </c>
       <c r="D16" s="7" t="inlineStr">
         <is>
-          <t>普卡基／Twizel</t>
+          <t>蒂阿瑙</t>
         </is>
       </c>
       <c r="E16" s="26" t="inlineStr">
         <is>
-          <t>Pukaki↔Mt Cook 往返 1.5h</t>
+          <t>Arrowtown→Te Anau 2.5h</t>
         </is>
       </c>
       <c r="F16" s="27" t="n">
-        <v>140</v>
+        <v>190</v>
       </c>
       <c r="G16" s="26" t="inlineStr">
         <is>
-          <t>庫克山一日：早上 Hooker Valley（免費必走），下午 Glacier Explorers 冰河湖船。</t>
+          <t>中午前出發。超市補米佛隔日食物。螢火蟲洞想去再訂。</t>
         </is>
       </c>
       <c r="H16" s="26" t="inlineStr">
         <is>
-          <t>庫克山 Glacier Explorers</t>
+          <t>—</t>
         </is>
       </c>
       <c r="I16" s="23" t="n">
-        <v>438</v>
+        <v>0</v>
       </c>
       <c r="J16" s="23" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="K16" s="23" t="n">
-        <v>140</v>
+        <v>130</v>
       </c>
       <c r="L16" s="23" t="n">
-        <v>30</v>
+        <v>42</v>
       </c>
       <c r="M16" s="28">
         <f>('01_總覽'!$B$8+'01_總覽'!$B$9)</f>
@@ -2253,116 +2253,116 @@
       </c>
       <c r="P16" s="26" t="inlineStr">
         <is>
-          <t>連住，看得到庫克山最好｜船是 NZ$219／人，從 2026/10/1。隱士只上去吃飯／報到，不必硬住。</t>
+          <t>Distinction / Lakefront｜螢火蟲洞約 NZ$145–154／人，累了就看湖。</t>
         </is>
       </c>
     </row>
     <row r="17" ht="48" customHeight="1">
-      <c r="A17" s="20" t="n">
+      <c r="A17" s="31" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="21" t="inlineStr">
+      <c r="B17" s="32" t="inlineStr">
         <is>
           <t>2027/5/1</t>
         </is>
       </c>
-      <c r="C17" s="21" t="inlineStr">
+      <c r="C17" s="32" t="inlineStr">
         <is>
           <t>六</t>
         </is>
       </c>
-      <c r="D17" s="21" t="inlineStr">
-        <is>
-          <t>蒂卡波</t>
-        </is>
-      </c>
-      <c r="E17" s="11" t="inlineStr">
-        <is>
-          <t>Pukaki→Tekapo 50min</t>
-        </is>
-      </c>
-      <c r="F17" s="22" t="n">
-        <v>70</v>
-      </c>
-      <c r="G17" s="11" t="inlineStr">
-        <is>
-          <t>普卡基再看一次日出。慢慢開到蒂卡波。下午湖邊、Tekapo Springs。教堂等人少再拍。</t>
-        </is>
-      </c>
-      <c r="H17" s="11" t="inlineStr">
-        <is>
-          <t>蒂卡波溫泉（可選）</t>
+      <c r="D17" s="32" t="inlineStr">
+        <is>
+          <t>蒂阿瑙</t>
+        </is>
+      </c>
+      <c r="E17" s="33" t="inlineStr">
+        <is>
+          <t>Te Anau↔Milford 往返 5h</t>
+        </is>
+      </c>
+      <c r="F17" s="34" t="n">
+        <v>240</v>
+      </c>
+      <c r="G17" s="33" t="inlineStr">
+        <is>
+          <t>07:00 自駕 SH94。訂 11:10 或 13:30 小船。傍晚回蒂阿瑙。</t>
+        </is>
+      </c>
+      <c r="H17" s="33" t="inlineStr">
+        <is>
+          <t>米佛峽灣遊船（自駕＋船）</t>
         </is>
       </c>
       <c r="I17" s="23" t="n">
-        <v>0</v>
+        <v>376</v>
       </c>
       <c r="J17" s="23" t="n">
-        <v>230</v>
+        <v>180</v>
       </c>
       <c r="K17" s="23" t="n">
         <v>130</v>
       </c>
       <c r="L17" s="23" t="n">
+        <v>52</v>
+      </c>
+      <c r="M17" s="35">
+        <f>('01_總覽'!$B$8+'01_總覽'!$B$9)</f>
+        <v/>
+      </c>
+      <c r="N17" s="36">
+        <f>I17+J17+K17+L17+M17</f>
+        <v/>
+      </c>
+      <c r="O17" s="37">
+        <f>N17*'01_總覽'!$B$5</f>
+        <v/>
+      </c>
+      <c r="P17" s="33" t="inlineStr">
+        <is>
+          <t>連住｜Mitre Peak／Cruise Milford 約 NZ$179–188。不要買皇后鎮巴士一日遊。</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="48" customHeight="1">
+      <c r="A18" s="31" t="n">
         <v>16</v>
       </c>
-      <c r="M17" s="12">
-        <f>('01_總覽'!$B$8+'01_總覽'!$B$9)</f>
-        <v/>
-      </c>
-      <c r="N17" s="24">
-        <f>I17+J17+K17+L17+M17</f>
-        <v/>
-      </c>
-      <c r="O17" s="13">
-        <f>N17*'01_總覽'!$B$5</f>
-        <v/>
-      </c>
-      <c r="P17" s="11" t="inlineStr">
-        <is>
-          <t>湖景 motel；無景房不值得｜牧羊人教堂日出比日落空。這兩晚就是發呆用的。</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="48" customHeight="1">
-      <c r="A18" s="25" t="n">
-        <v>16</v>
-      </c>
-      <c r="B18" s="7" t="inlineStr">
+      <c r="B18" s="32" t="inlineStr">
         <is>
           <t>2027/5/2</t>
         </is>
       </c>
-      <c r="C18" s="7" t="inlineStr">
+      <c r="C18" s="32" t="inlineStr">
         <is>
           <t>日</t>
         </is>
       </c>
-      <c r="D18" s="7" t="inlineStr">
+      <c r="D18" s="32" t="inlineStr">
         <is>
           <t>蒂卡波</t>
         </is>
       </c>
-      <c r="E18" s="26" t="inlineStr">
-        <is>
-          <t>當地</t>
-        </is>
-      </c>
-      <c r="F18" s="27" t="n">
-        <v>25</v>
-      </c>
-      <c r="G18" s="26" t="inlineStr">
-        <is>
-          <t>整天留著。想觀星就訂 Dark Sky 約翰山 Summit；雲多可改 Crater 或自己看。</t>
-        </is>
-      </c>
-      <c r="H18" s="26" t="inlineStr">
-        <is>
-          <t>Dark Sky 約翰山 Summit</t>
+      <c r="E18" s="33" t="inlineStr">
+        <is>
+          <t>Te Anau→Tekapo 6h</t>
+        </is>
+      </c>
+      <c r="F18" s="34" t="n">
+        <v>400</v>
+      </c>
+      <c r="G18" s="33" t="inlineStr">
+        <is>
+          <t>經 Cromwell、Lindis 回麥肯齊。傍晚到蒂卡波，不排觀星。</t>
+        </is>
+      </c>
+      <c r="H18" s="33" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="I18" s="23" t="n">
-        <v>478</v>
+        <v>0</v>
       </c>
       <c r="J18" s="23" t="n">
         <v>230</v>
@@ -2371,23 +2371,23 @@
         <v>130</v>
       </c>
       <c r="L18" s="23" t="n">
-        <v>6</v>
-      </c>
-      <c r="M18" s="28">
+        <v>85</v>
+      </c>
+      <c r="M18" s="35">
         <f>('01_總覽'!$B$8+'01_總覽'!$B$9)</f>
         <v/>
       </c>
-      <c r="N18" s="29">
+      <c r="N18" s="36">
         <f>I18+J18+K18+L18+M18</f>
         <v/>
       </c>
-      <c r="O18" s="30">
+      <c r="O18" s="37">
         <f>N18*'01_總覽'!$B$5</f>
         <v/>
       </c>
-      <c r="P18" s="26" t="inlineStr">
-        <is>
-          <t>連住第 2 晚｜Summit 約 NZ$219–239。天氣不好有室內備援。</t>
+      <c r="P18" s="33" t="inlineStr">
+        <is>
+          <t>湖景 motel｜米佛隔天不要直接開回基督城，那是 8 小時以上。</t>
         </is>
       </c>
     </row>
@@ -2420,7 +2420,7 @@
       </c>
       <c r="G19" s="11" t="inlineStr">
         <is>
-          <t>上午離開。還車前加滿油。住機場附近。有力氣才去阿卡羅阿看企鵝，不排進預算。</t>
+          <t>上午離開。還車前加滿油。住機場附近。</t>
         </is>
       </c>
       <c r="H19" s="11" t="inlineStr">
@@ -2723,24 +2723,24 @@
     <row r="5">
       <c r="A5" s="40" t="inlineStr">
         <is>
-          <t>霍基蒂卡</t>
+          <t>蒂卡波（去程）</t>
         </is>
       </c>
       <c r="B5" s="41" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="C5" s="21" t="inlineStr">
         <is>
-          <t>4/20</t>
+          <t>4/20–21</t>
         </is>
       </c>
       <c r="D5" s="11" t="inlineStr">
         <is>
-          <t>中價 motel</t>
+          <t>湖景</t>
         </is>
       </c>
       <c r="E5" s="23" t="n">
-        <v>140</v>
+        <v>230</v>
       </c>
       <c r="F5" s="24">
         <f>B5*E5</f>
@@ -2752,14 +2752,14 @@
       </c>
       <c r="H5" s="11" t="inlineStr">
         <is>
-          <t>拆開西岸長途</t>
+          <t>教堂＋觀星</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="42" t="inlineStr">
         <is>
-          <t>弗蘭茲約瑟夫</t>
+          <t>庫克山村</t>
         </is>
       </c>
       <c r="B6" s="43" t="n">
@@ -2767,16 +2767,16 @@
       </c>
       <c r="C6" s="7" t="inlineStr">
         <is>
-          <t>4/21–23</t>
+          <t>4/22–24</t>
         </is>
       </c>
       <c r="D6" s="26" t="inlineStr">
         <is>
-          <t>村內 motel</t>
+          <t>隱士山景或 Aoraki Court</t>
         </is>
       </c>
       <c r="E6" s="23" t="n">
-        <v>180</v>
+        <v>320</v>
       </c>
       <c r="F6" s="29">
         <f>B6*E6</f>
@@ -2788,31 +2788,31 @@
       </c>
       <c r="H6" s="26" t="inlineStr">
         <is>
-          <t>冰川天氣緩衝</t>
+          <t>塔斯曼冰川就在村外，天氣緩衝</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="40" t="inlineStr">
         <is>
-          <t>箭鎮</t>
+          <t>普卡基／Twizel</t>
         </is>
       </c>
       <c r="B7" s="41" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="C7" s="21" t="inlineStr">
         <is>
-          <t>4/24–26</t>
+          <t>4/25–26</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>村內、能走去主街</t>
+          <t>能看庫克山的 cabin</t>
         </is>
       </c>
       <c r="E7" s="23" t="n">
-        <v>230</v>
+        <v>200</v>
       </c>
       <c r="F7" s="24">
         <f>B7*E7</f>
@@ -2824,31 +2824,31 @@
       </c>
       <c r="H7" s="11" t="inlineStr">
         <is>
-          <t>楓葉季住村裡，清晨沒人</t>
+          <t>湖邊久住</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="42" t="inlineStr">
         <is>
-          <t>蒂阿瑙</t>
+          <t>箭鎮</t>
         </is>
       </c>
       <c r="B8" s="43" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="C8" s="7" t="inlineStr">
         <is>
-          <t>4/27–28</t>
+          <t>4/27–29</t>
         </is>
       </c>
       <c r="D8" s="26" t="inlineStr">
         <is>
-          <t>湖濱 motel</t>
+          <t>村內、能走去主街</t>
         </is>
       </c>
       <c r="E8" s="23" t="n">
-        <v>180</v>
+        <v>230</v>
       </c>
       <c r="F8" s="29">
         <f>B8*E8</f>
@@ -2860,14 +2860,14 @@
       </c>
       <c r="H8" s="26" t="inlineStr">
         <is>
-          <t>米佛自駕基地</t>
+          <t>楓葉季住村裡</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="40" t="inlineStr">
         <is>
-          <t>普卡基／Twizel</t>
+          <t>蒂阿瑙</t>
         </is>
       </c>
       <c r="B9" s="41" t="n">
@@ -2875,16 +2875,16 @@
       </c>
       <c r="C9" s="21" t="inlineStr">
         <is>
-          <t>4/29–30</t>
+          <t>4/30–5/1</t>
         </is>
       </c>
       <c r="D9" s="11" t="inlineStr">
         <is>
-          <t>能看庫克山的 cabin／motel</t>
+          <t>湖濱 motel</t>
         </is>
       </c>
       <c r="E9" s="23" t="n">
-        <v>200</v>
+        <v>180</v>
       </c>
       <c r="F9" s="24">
         <f>B9*E9</f>
@@ -2896,22 +2896,22 @@
       </c>
       <c r="H9" s="11" t="inlineStr">
         <is>
-          <t>庫克山一日來回，比隱士便宜</t>
+          <t>米佛自駕基地</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="42" t="inlineStr">
         <is>
-          <t>蒂卡波</t>
+          <t>蒂卡波（回程）</t>
         </is>
       </c>
       <c r="B10" s="43" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="C10" s="7" t="inlineStr">
         <is>
-          <t>5/1–2</t>
+          <t>5/2</t>
         </is>
       </c>
       <c r="D10" s="26" t="inlineStr">
@@ -2932,7 +2932,7 @@
       </c>
       <c r="H10" s="26" t="inlineStr">
         <is>
-          <t>教堂＋觀星，無景房不要</t>
+          <t>拆開回基督城的長途</t>
         </is>
       </c>
     </row>
@@ -3219,7 +3219,7 @@
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>含米佛往返、庫克山一日。</t>
+          <t>不含西岸。含米佛往返。</t>
         </is>
       </c>
     </row>
@@ -3373,7 +3373,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:F15"/>
+  <dimension ref="A1:F13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -3454,16 +3454,16 @@
     <row r="4">
       <c r="A4" s="7" t="inlineStr">
         <is>
-          <t>D4 4/20</t>
+          <t>D5 4/21</t>
         </is>
       </c>
       <c r="B4" s="42" t="inlineStr">
         <is>
-          <t>漢默泉泡湯（可選）</t>
+          <t>Dark Sky 約翰山 Summit</t>
         </is>
       </c>
       <c r="C4" s="23" t="n">
-        <v>40</v>
+        <v>239</v>
       </c>
       <c r="D4" s="28">
         <f>C4*'01_總覽'!$B$4</f>
@@ -3475,23 +3475,23 @@
       </c>
       <c r="F4" s="26" t="inlineStr">
         <is>
-          <t>中途休息，不必過夜。官網約 NZ$38–42。</t>
+          <t>官網 219–239。可改 Crater NZ$129。</t>
         </is>
       </c>
     </row>
     <row r="5">
       <c r="A5" s="21" t="inlineStr">
         <is>
-          <t>D6 4/22</t>
+          <t>D7 4/23</t>
         </is>
       </c>
       <c r="B5" s="40" t="inlineStr">
         <is>
-          <t>Franz Josef heli-hike</t>
+          <t>Tasman Glacier heli-hike</t>
         </is>
       </c>
       <c r="C5" s="23" t="n">
-        <v>899</v>
+        <v>995</v>
       </c>
       <c r="D5" s="12">
         <f>C5*'01_總覽'!$B$4</f>
@@ -3503,14 +3503,14 @@
       </c>
       <c r="F5" s="11" t="inlineStr">
         <is>
-          <t>官網至 2027/9/30。4/23 當備援。</t>
+          <t>庫克山機場出發。Alpine Guides／Mt Cook Glacier Guiding 至 2027/9/30。4/24 備援。</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>D12 4/28</t>
+          <t>D15 5/1</t>
         </is>
       </c>
       <c r="B6" s="42" t="inlineStr">
@@ -3536,107 +3536,81 @@
       </c>
     </row>
     <row r="7">
-      <c r="A7" s="21" t="inlineStr">
-        <is>
-          <t>D14 4/30</t>
-        </is>
-      </c>
-      <c r="B7" s="40" t="inlineStr">
-        <is>
-          <t>庫克山 Glacier Explorers</t>
-        </is>
-      </c>
-      <c r="C7" s="23" t="n">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="B7" s="5" t="n"/>
+      <c r="C7" s="14">
+        <f>SUM(C3:C6)</f>
+        <v/>
+      </c>
+      <c r="D7" s="14">
+        <f>SUM(D3:D6)</f>
+        <v/>
+      </c>
+      <c r="E7" s="15">
+        <f>D7*'01_總覽'!$B$5</f>
+        <v/>
+      </c>
+      <c r="F7" s="47" t="inlineStr">
+        <is>
+          <t>冰川健行在庫克山，不是弗蘭茲</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>這次故意沒排、想加再加</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="10" t="inlineStr">
+        <is>
+          <t>可選</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>一人 NZD</t>
+        </is>
+      </c>
+      <c r="C10" s="10" t="inlineStr">
+        <is>
+          <t>怎麼加</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>Tasman Glacier View 步道</t>
+        </is>
+      </c>
+      <c r="B11" s="12" t="n">
+        <v>0</v>
+      </c>
+      <c r="C11" s="11" t="inlineStr">
+        <is>
+          <t>村外開車 10 分，免費看冰川末端。走不上冰。</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>Glacier Explorers 冰河湖船</t>
+        </is>
+      </c>
+      <c r="B12" s="12" t="n">
         <v>219</v>
       </c>
-      <c r="D7" s="12">
-        <f>C7*'01_總覽'!$B$4</f>
-        <v/>
-      </c>
-      <c r="E7" s="13">
-        <f>D7*'01_總覽'!$B$5</f>
-        <v/>
-      </c>
-      <c r="F7" s="11" t="inlineStr">
-        <is>
-          <t>2026/10/1 起 NZ$219。不要訂成 Tasman heli-hike。</t>
-        </is>
-      </c>
-    </row>
-    <row r="8">
-      <c r="A8" s="7" t="inlineStr">
-        <is>
-          <t>D16 5/2</t>
-        </is>
-      </c>
-      <c r="B8" s="42" t="inlineStr">
-        <is>
-          <t>Dark Sky 約翰山 Summit</t>
-        </is>
-      </c>
-      <c r="C8" s="23" t="n">
-        <v>239</v>
-      </c>
-      <c r="D8" s="28">
-        <f>C8*'01_總覽'!$B$4</f>
-        <v/>
-      </c>
-      <c r="E8" s="30">
-        <f>D8*'01_總覽'!$B$5</f>
-        <v/>
-      </c>
-      <c r="F8" s="26" t="inlineStr">
-        <is>
-          <t>官網 219–239。可改 Crater NZ$129。</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="5" t="inlineStr">
-        <is>
-          <t>合計</t>
-        </is>
-      </c>
-      <c r="B9" s="5" t="n"/>
-      <c r="C9" s="14">
-        <f>SUM(C3:C8)</f>
-        <v/>
-      </c>
-      <c r="D9" s="14">
-        <f>SUM(D3:D8)</f>
-        <v/>
-      </c>
-      <c r="E9" s="15">
-        <f>D9*'01_總覽'!$B$5</f>
-        <v/>
-      </c>
-      <c r="F9" s="47" t="inlineStr">
-        <is>
-          <t>漢默若不去，把 D4 活動改 0</t>
-        </is>
-      </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="4" t="inlineStr">
-        <is>
-          <t>這次故意沒排、想加再加</t>
-        </is>
-      </c>
-    </row>
-    <row r="12">
-      <c r="A12" s="10" t="inlineStr">
-        <is>
-          <t>可選</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
-        <is>
-          <t>一人 NZD</t>
-        </is>
-      </c>
-      <c r="C12" s="10" t="inlineStr">
-        <is>
-          <t>怎麼加</t>
+      <c r="C12" s="11" t="inlineStr">
+        <is>
+          <t>隱士一樓報到。是坐船看冰山，不是冰川健行。</t>
         </is>
       </c>
     </row>
@@ -3651,37 +3625,7 @@
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>D11 晚上。累了就睡。</t>
-        </is>
-      </c>
-    </row>
-    <row r="14">
-      <c r="A14" s="11" t="inlineStr">
-        <is>
-          <t>奧瑪魯小藍企鵝</t>
-        </is>
-      </c>
-      <c r="B14" s="12" t="n">
-        <v>70</v>
-      </c>
-      <c r="C14" s="11" t="inlineStr">
-        <is>
-          <t>這條 chill 線不繞東岸。若很想看，5/3 改阿卡羅阿 Pohatu。</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" s="11" t="inlineStr">
-        <is>
-          <t>隱士飯店山景 1 晚</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="n">
-        <v>340</v>
-      </c>
-      <c r="C15" s="11" t="inlineStr">
-        <is>
-          <t>普卡基已能看庫克山。只想住一次再把 D14 改住隱士。</t>
+          <t>4/30 晚上。累了就睡。</t>
         </is>
       </c>
     </row>
@@ -3970,25 +3914,25 @@
       </c>
       <c r="C6" s="32" t="inlineStr">
         <is>
-          <t>霍基蒂卡</t>
+          <t>蒂卡波</t>
         </is>
       </c>
       <c r="D6" s="33" t="inlineStr">
         <is>
-          <t>經 Hanmer＋Lewis Pass 6.5h</t>
+          <t>Kaikoura→Tekapo 6h</t>
         </is>
       </c>
       <c r="E6" s="48" t="n">
-        <v>420</v>
+        <v>450</v>
       </c>
       <c r="F6" s="33" t="inlineStr">
         <is>
-          <t>經漢默泉泡湯 1.5–2h（不必過夜），再走 Lewis Pass 到西岸。夠力再停 Pancake Rocks。</t>
+          <t>原路回 SH1 南下，經 Geraldine、Fairlie 進麥肯齊。傍晚牧羊人教堂。不繞西岸。</t>
         </is>
       </c>
       <c r="G6" s="32" t="inlineStr">
         <is>
-          <t>漢默泉泡湯（可選）</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H6" s="23">
@@ -4027,25 +3971,25 @@
       </c>
       <c r="C7" s="21" t="inlineStr">
         <is>
-          <t>弗蘭茲約瑟夫</t>
+          <t>蒂卡波</t>
         </is>
       </c>
       <c r="D7" s="11" t="inlineStr">
         <is>
-          <t>Hokitika→Franz 2h</t>
+          <t>當地</t>
         </is>
       </c>
       <c r="E7" s="41" t="n">
-        <v>160</v>
+        <v>25</v>
       </c>
       <c r="F7" s="11" t="inlineStr">
         <is>
-          <t>上午 Hokitika Gorge（免費、水色很美）。午後抵冰川村報到、走谷底步道遠看冰。</t>
+          <t>整天留著。教堂日出、湖邊、Tekapo Springs。晚上 Dark Sky 約翰山。</t>
         </is>
       </c>
       <c r="G7" s="21" t="inlineStr">
         <is>
-          <t>—</t>
+          <t>Dark Sky 約翰山 Summit</t>
         </is>
       </c>
       <c r="H7" s="23">
@@ -4074,35 +4018,35 @@
       </c>
     </row>
     <row r="8" ht="36" customHeight="1">
-      <c r="A8" s="32" t="n">
+      <c r="A8" s="21" t="n">
         <v>6</v>
       </c>
-      <c r="B8" s="32" t="inlineStr">
+      <c r="B8" s="21" t="inlineStr">
         <is>
           <t>2027/4/22 四</t>
         </is>
       </c>
-      <c r="C8" s="32" t="inlineStr">
-        <is>
-          <t>弗蘭茲約瑟夫</t>
-        </is>
-      </c>
-      <c r="D8" s="33" t="inlineStr">
-        <is>
-          <t>當地</t>
-        </is>
-      </c>
-      <c r="E8" s="48" t="n">
-        <v>20</v>
-      </c>
-      <c r="F8" s="33" t="inlineStr">
-        <is>
-          <t>直升機冰川健行（半天，裝備全含）。取消則改 4/23。下午回房休息。</t>
-        </is>
-      </c>
-      <c r="G8" s="32" t="inlineStr">
-        <is>
-          <t>Franz heli-hike</t>
+      <c r="C8" s="21" t="inlineStr">
+        <is>
+          <t>庫克山村</t>
+        </is>
+      </c>
+      <c r="D8" s="11" t="inlineStr">
+        <is>
+          <t>Tekapo→Mt Cook 1.5h</t>
+        </is>
+      </c>
+      <c r="E8" s="41" t="n">
+        <v>105</v>
+      </c>
+      <c r="F8" s="11" t="inlineStr">
+        <is>
+          <t>經普卡基牛奶藍進村。下午走免費 Tasman Glacier View（車 10 分＋步道 40 分）。報到冰川健行。</t>
+        </is>
+      </c>
+      <c r="G8" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H8" s="23">
@@ -4121,45 +4065,45 @@
         <f>'02_每日行程'!L8</f>
         <v/>
       </c>
-      <c r="L8" s="35">
+      <c r="L8" s="12">
         <f>'02_每日行程'!M8</f>
         <v/>
       </c>
-      <c r="M8" s="35">
+      <c r="M8" s="12">
         <f>'02_每日行程'!N8</f>
         <v/>
       </c>
     </row>
     <row r="9" ht="36" customHeight="1">
-      <c r="A9" s="21" t="n">
+      <c r="A9" s="32" t="n">
         <v>7</v>
       </c>
-      <c r="B9" s="21" t="inlineStr">
+      <c r="B9" s="32" t="inlineStr">
         <is>
           <t>2027/4/23 五</t>
         </is>
       </c>
-      <c r="C9" s="21" t="inlineStr">
-        <is>
-          <t>弗蘭茲約瑟夫</t>
-        </is>
-      </c>
-      <c r="D9" s="11" t="inlineStr">
-        <is>
-          <t>Franz↔Fox 往返</t>
-        </is>
-      </c>
-      <c r="E9" s="41" t="n">
-        <v>50</v>
-      </c>
-      <c r="F9" s="11" t="inlineStr">
-        <is>
-          <t>天氣備援日。能飛就補 heli-hike；不能就黎明去 Lake Matheson 拍鏡面。整天可以很閒。</t>
-        </is>
-      </c>
-      <c r="G9" s="21" t="inlineStr">
-        <is>
-          <t>—</t>
+      <c r="C9" s="32" t="inlineStr">
+        <is>
+          <t>庫克山村</t>
+        </is>
+      </c>
+      <c r="D9" s="33" t="inlineStr">
+        <is>
+          <t>當地／機場 10 分</t>
+        </is>
+      </c>
+      <c r="E9" s="48" t="n">
+        <v>20</v>
+      </c>
+      <c r="F9" s="33" t="inlineStr">
+        <is>
+          <t>塔斯曼冰川健行：庫克山機場集合，直升機上冰走約 2 小時。取消則改 4/24。</t>
+        </is>
+      </c>
+      <c r="G9" s="32" t="inlineStr">
+        <is>
+          <t>Tasman Glacier heli-hike</t>
         </is>
       </c>
       <c r="H9" s="23">
@@ -4178,43 +4122,43 @@
         <f>'02_每日行程'!L9</f>
         <v/>
       </c>
-      <c r="L9" s="12">
+      <c r="L9" s="35">
         <f>'02_每日行程'!M9</f>
         <v/>
       </c>
-      <c r="M9" s="12">
+      <c r="M9" s="35">
         <f>'02_每日行程'!N9</f>
         <v/>
       </c>
     </row>
     <row r="10" ht="36" customHeight="1">
-      <c r="A10" s="32" t="n">
+      <c r="A10" s="21" t="n">
         <v>8</v>
       </c>
-      <c r="B10" s="32" t="inlineStr">
+      <c r="B10" s="21" t="inlineStr">
         <is>
           <t>2027/4/24 六</t>
         </is>
       </c>
-      <c r="C10" s="32" t="inlineStr">
-        <is>
-          <t>箭鎮</t>
-        </is>
-      </c>
-      <c r="D10" s="33" t="inlineStr">
-        <is>
-          <t>Franz→Haast→Wanaka→Arrowtown 5h</t>
-        </is>
-      </c>
-      <c r="E10" s="48" t="n">
-        <v>400</v>
-      </c>
-      <c r="F10" s="33" t="inlineStr">
-        <is>
-          <t>Haast Pass 本身是景。Wanaka 咖啡＋That Wanaka Tree。傍晚進箭鎮住下來。</t>
-        </is>
-      </c>
-      <c r="G10" s="32" t="inlineStr">
+      <c r="C10" s="21" t="inlineStr">
+        <is>
+          <t>庫克山村</t>
+        </is>
+      </c>
+      <c r="D10" s="11" t="inlineStr">
+        <is>
+          <t>當地</t>
+        </is>
+      </c>
+      <c r="E10" s="41" t="n">
+        <v>25</v>
+      </c>
+      <c r="F10" s="11" t="inlineStr">
+        <is>
+          <t>天氣備援日。能飛就補健行；不能就走 Hooker Valley。想坐冰河湖船再加 Glacier Explorers。</t>
+        </is>
+      </c>
+      <c r="G10" s="21" t="inlineStr">
         <is>
           <t>—</t>
         </is>
@@ -4235,11 +4179,11 @@
         <f>'02_每日行程'!L10</f>
         <v/>
       </c>
-      <c r="L10" s="35">
+      <c r="L10" s="12">
         <f>'02_每日行程'!M10</f>
         <v/>
       </c>
-      <c r="M10" s="35">
+      <c r="M10" s="12">
         <f>'02_每日行程'!N10</f>
         <v/>
       </c>
@@ -4255,20 +4199,20 @@
       </c>
       <c r="C11" s="21" t="inlineStr">
         <is>
-          <t>箭鎮</t>
+          <t>普卡基／Twizel</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
         <is>
-          <t>當地／Lake Hayes</t>
+          <t>Mt Cook→Pukaki 50min</t>
         </is>
       </c>
       <c r="E11" s="41" t="n">
-        <v>40</v>
+        <v>70</v>
       </c>
       <c r="F11" s="11" t="inlineStr">
         <is>
-          <t>07:30 前走 Buckingham Street、中國村、Arrow River。再到 Lake Hayes 拍倒影。下午發呆。</t>
+          <t>早上 Hooker Valley（若昨天沒走）。慢慢開到普卡基看牛奶藍，下午發呆。</t>
         </is>
       </c>
       <c r="G11" s="21" t="inlineStr">
@@ -4312,20 +4256,20 @@
       </c>
       <c r="C12" s="21" t="inlineStr">
         <is>
-          <t>箭鎮</t>
+          <t>普卡基／Twizel</t>
         </is>
       </c>
       <c r="D12" s="11" t="inlineStr">
         <is>
-          <t>可去皇后鎮或 Glenorchy</t>
+          <t>當地</t>
         </is>
       </c>
       <c r="E12" s="41" t="n">
-        <v>80</v>
+        <v>40</v>
       </c>
       <c r="F12" s="11" t="inlineStr">
         <is>
-          <t>週一比較空。可去 Glenorchy 湖灣，或皇后鎮散步。不跳傘、不彈跳。酒莊要有指定駕駛。</t>
+          <t>整天留著。日出看庫克山、沿湖散步。不想開車就待著。</t>
         </is>
       </c>
       <c r="G12" s="21" t="inlineStr">
@@ -4369,25 +4313,25 @@
       </c>
       <c r="C13" s="21" t="inlineStr">
         <is>
-          <t>蒂阿瑙</t>
+          <t>箭鎮</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
         <is>
-          <t>Arrowtown→Te Anau 2.5h</t>
+          <t>Pukaki→Lindis→Arrowtown 4h</t>
         </is>
       </c>
       <c r="E13" s="41" t="n">
-        <v>190</v>
+        <v>280</v>
       </c>
       <c r="F13" s="11" t="inlineStr">
         <is>
-          <t>中午前出發即可。超市補米佛隔日食物（沿路沒店）。晚上想去再訂螢火蟲洞，不勉強。</t>
+          <t>經 Omarama、Lindis Pass、Cromwell。Wanaka 想停就停。傍晚進箭鎮。</t>
         </is>
       </c>
       <c r="G13" s="21" t="inlineStr">
         <is>
-          <t>螢火蟲洞（可選，表內未列）</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H13" s="23">
@@ -4416,35 +4360,35 @@
       </c>
     </row>
     <row r="14" ht="36" customHeight="1">
-      <c r="A14" s="32" t="n">
+      <c r="A14" s="21" t="n">
         <v>12</v>
       </c>
-      <c r="B14" s="32" t="inlineStr">
+      <c r="B14" s="21" t="inlineStr">
         <is>
           <t>2027/4/28 三</t>
         </is>
       </c>
-      <c r="C14" s="32" t="inlineStr">
-        <is>
-          <t>蒂阿瑙</t>
-        </is>
-      </c>
-      <c r="D14" s="33" t="inlineStr">
-        <is>
-          <t>Te Anau↔Milford 往返 5h</t>
-        </is>
-      </c>
-      <c r="E14" s="48" t="n">
-        <v>240</v>
-      </c>
-      <c r="F14" s="33" t="inlineStr">
-        <is>
-          <t>07:00 自駕 SH94：Mirror Lakes、Homer Tunnel。訂 11:10 或 13:30 小船。傍晚回蒂阿瑙。</t>
-        </is>
-      </c>
-      <c r="G14" s="32" t="inlineStr">
-        <is>
-          <t>米佛峽灣遊船（自駕＋船）</t>
+      <c r="C14" s="21" t="inlineStr">
+        <is>
+          <t>箭鎮</t>
+        </is>
+      </c>
+      <c r="D14" s="11" t="inlineStr">
+        <is>
+          <t>當地／Lake Hayes</t>
+        </is>
+      </c>
+      <c r="E14" s="41" t="n">
+        <v>40</v>
+      </c>
+      <c r="F14" s="11" t="inlineStr">
+        <is>
+          <t>07:30 前走 Buckingham Street、中國村、Arrow River。再到 Lake Hayes。</t>
+        </is>
+      </c>
+      <c r="G14" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H14" s="23">
@@ -4463,45 +4407,45 @@
         <f>'02_每日行程'!L14</f>
         <v/>
       </c>
-      <c r="L14" s="35">
+      <c r="L14" s="12">
         <f>'02_每日行程'!M14</f>
         <v/>
       </c>
-      <c r="M14" s="35">
+      <c r="M14" s="12">
         <f>'02_每日行程'!N14</f>
         <v/>
       </c>
     </row>
     <row r="15" ht="36" customHeight="1">
-      <c r="A15" s="32" t="n">
+      <c r="A15" s="21" t="n">
         <v>13</v>
       </c>
-      <c r="B15" s="32" t="inlineStr">
+      <c r="B15" s="21" t="inlineStr">
         <is>
           <t>2027/4/29 四</t>
         </is>
       </c>
-      <c r="C15" s="32" t="inlineStr">
-        <is>
-          <t>普卡基／Twizel</t>
-        </is>
-      </c>
-      <c r="D15" s="33" t="inlineStr">
-        <is>
-          <t>經 Cromwell＋Lindis 6h</t>
-        </is>
-      </c>
-      <c r="E15" s="48" t="n">
-        <v>400</v>
-      </c>
-      <c r="F15" s="33" t="inlineStr">
-        <is>
-          <t>回程不繞但尼丁。Lindis Pass 秋天很美。Omarama 可停熱湯池。傍晚抵普卡基看牛奶藍。</t>
-        </is>
-      </c>
-      <c r="G15" s="32" t="inlineStr">
-        <is>
-          <t>Omarama Hot Tubs（可選）</t>
+      <c r="C15" s="21" t="inlineStr">
+        <is>
+          <t>箭鎮</t>
+        </is>
+      </c>
+      <c r="D15" s="11" t="inlineStr">
+        <is>
+          <t>可去 Glenorchy</t>
+        </is>
+      </c>
+      <c r="E15" s="41" t="n">
+        <v>80</v>
+      </c>
+      <c r="F15" s="11" t="inlineStr">
+        <is>
+          <t>人少的一天。Glenorchy 湖灣或皇后鎮散步。不跳傘。</t>
+        </is>
+      </c>
+      <c r="G15" s="21" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H15" s="23">
@@ -4520,11 +4464,11 @@
         <f>'02_每日行程'!L15</f>
         <v/>
       </c>
-      <c r="L15" s="35">
+      <c r="L15" s="12">
         <f>'02_每日行程'!M15</f>
         <v/>
       </c>
-      <c r="M15" s="35">
+      <c r="M15" s="12">
         <f>'02_每日行程'!N15</f>
         <v/>
       </c>
@@ -4540,25 +4484,25 @@
       </c>
       <c r="C16" s="21" t="inlineStr">
         <is>
-          <t>普卡基／Twizel</t>
+          <t>蒂阿瑙</t>
         </is>
       </c>
       <c r="D16" s="11" t="inlineStr">
         <is>
-          <t>Pukaki↔Mt Cook 往返 1.5h</t>
+          <t>Arrowtown→Te Anau 2.5h</t>
         </is>
       </c>
       <c r="E16" s="41" t="n">
-        <v>140</v>
+        <v>190</v>
       </c>
       <c r="F16" s="11" t="inlineStr">
         <is>
-          <t>庫克山一日：早上 Hooker Valley（免費必走），下午 Glacier Explorers 冰河湖船。</t>
+          <t>中午前出發。超市補米佛隔日食物。螢火蟲洞想去再訂。</t>
         </is>
       </c>
       <c r="G16" s="21" t="inlineStr">
         <is>
-          <t>庫克山 Glacier Explorers</t>
+          <t>—</t>
         </is>
       </c>
       <c r="H16" s="23">
@@ -4587,35 +4531,35 @@
       </c>
     </row>
     <row r="17" ht="36" customHeight="1">
-      <c r="A17" s="21" t="n">
+      <c r="A17" s="32" t="n">
         <v>15</v>
       </c>
-      <c r="B17" s="21" t="inlineStr">
+      <c r="B17" s="32" t="inlineStr">
         <is>
           <t>2027/5/1 六</t>
         </is>
       </c>
-      <c r="C17" s="21" t="inlineStr">
-        <is>
-          <t>蒂卡波</t>
-        </is>
-      </c>
-      <c r="D17" s="11" t="inlineStr">
-        <is>
-          <t>Pukaki→Tekapo 50min</t>
-        </is>
-      </c>
-      <c r="E17" s="41" t="n">
-        <v>70</v>
-      </c>
-      <c r="F17" s="11" t="inlineStr">
-        <is>
-          <t>普卡基再看一次日出。慢慢開到蒂卡波。下午湖邊、Tekapo Springs。教堂等人少再拍。</t>
-        </is>
-      </c>
-      <c r="G17" s="21" t="inlineStr">
-        <is>
-          <t>蒂卡波溫泉（可選）</t>
+      <c r="C17" s="32" t="inlineStr">
+        <is>
+          <t>蒂阿瑙</t>
+        </is>
+      </c>
+      <c r="D17" s="33" t="inlineStr">
+        <is>
+          <t>Te Anau↔Milford 往返 5h</t>
+        </is>
+      </c>
+      <c r="E17" s="48" t="n">
+        <v>240</v>
+      </c>
+      <c r="F17" s="33" t="inlineStr">
+        <is>
+          <t>07:00 自駕 SH94。訂 11:10 或 13:30 小船。傍晚回蒂阿瑙。</t>
+        </is>
+      </c>
+      <c r="G17" s="32" t="inlineStr">
+        <is>
+          <t>米佛峽灣遊船（自駕＋船）</t>
         </is>
       </c>
       <c r="H17" s="23">
@@ -4634,45 +4578,45 @@
         <f>'02_每日行程'!L17</f>
         <v/>
       </c>
-      <c r="L17" s="12">
+      <c r="L17" s="35">
         <f>'02_每日行程'!M17</f>
         <v/>
       </c>
-      <c r="M17" s="12">
+      <c r="M17" s="35">
         <f>'02_每日行程'!N17</f>
         <v/>
       </c>
     </row>
     <row r="18" ht="36" customHeight="1">
-      <c r="A18" s="21" t="n">
+      <c r="A18" s="32" t="n">
         <v>16</v>
       </c>
-      <c r="B18" s="21" t="inlineStr">
+      <c r="B18" s="32" t="inlineStr">
         <is>
           <t>2027/5/2 日</t>
         </is>
       </c>
-      <c r="C18" s="21" t="inlineStr">
+      <c r="C18" s="32" t="inlineStr">
         <is>
           <t>蒂卡波</t>
         </is>
       </c>
-      <c r="D18" s="11" t="inlineStr">
-        <is>
-          <t>當地</t>
-        </is>
-      </c>
-      <c r="E18" s="41" t="n">
-        <v>25</v>
-      </c>
-      <c r="F18" s="11" t="inlineStr">
-        <is>
-          <t>整天留著。想觀星就訂 Dark Sky 約翰山 Summit；雲多可改 Crater 或自己看。</t>
-        </is>
-      </c>
-      <c r="G18" s="21" t="inlineStr">
-        <is>
-          <t>Dark Sky 約翰山 Summit</t>
+      <c r="D18" s="33" t="inlineStr">
+        <is>
+          <t>Te Anau→Tekapo 6h</t>
+        </is>
+      </c>
+      <c r="E18" s="48" t="n">
+        <v>400</v>
+      </c>
+      <c r="F18" s="33" t="inlineStr">
+        <is>
+          <t>經 Cromwell、Lindis 回麥肯齊。傍晚到蒂卡波，不排觀星。</t>
+        </is>
+      </c>
+      <c r="G18" s="32" t="inlineStr">
+        <is>
+          <t>—</t>
         </is>
       </c>
       <c r="H18" s="23">
@@ -4691,11 +4635,11 @@
         <f>'02_每日行程'!L18</f>
         <v/>
       </c>
-      <c r="L18" s="12">
+      <c r="L18" s="35">
         <f>'02_每日行程'!M18</f>
         <v/>
       </c>
-      <c r="M18" s="12">
+      <c r="M18" s="35">
         <f>'02_每日行程'!N18</f>
         <v/>
       </c>
@@ -4724,7 +4668,7 @@
       </c>
       <c r="F19" s="11" t="inlineStr">
         <is>
-          <t>上午離開。還車前加滿油。住機場附近。有力氣才去阿卡羅阿看企鵝，不排進預算。</t>
+          <t>上午離開。還車前加滿油。住機場附近。</t>
         </is>
       </c>
       <c r="G19" s="21" t="inlineStr">

</xml_diff>